<commit_message>
Integrate database-backed device/user features
Switch app data from hardcoded lists to Supabase-backed queries and add UI refinements. Adds .streamlit theme config and a new api.py stub, removes test.py. database.py: fix delete_device table, add typing import, implement delete_user, get_username, search_devices, total_devices and all_devices_name helpers to enable dynamic queries. main.py: refactor header layout, pull users and device names from database, use database.search_devices for listings, update badges to show serial, name, assigned user and purchase date, and adjust various UI behaviors (removed reruns and placeholder status handlers). Minor binary and pyc files changed/updated.
</commit_message>
<xml_diff>
--- a/Documentations/Planning-Journal_de_travail-TPI-Jimmy.xlsx
+++ b/Documentations/Planning-Journal_de_travail-TPI-Jimmy.xlsx
@@ -3,22 +3,22 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5F68F5E-E63D-44CB-AC79-E198D2B3BC13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{324D871E-12D2-4654-B26A-53DCCB56C5A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="21690" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planificateur de projet" sheetId="1" r:id="rId1"/>
     <sheet name="Journal de travail" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Planificateur de projet'!$3:$4</definedName>
     <definedName name="période_sélectionnée">'Planificateur de projet'!$H$2</definedName>
     <definedName name="PériodeDansPlan">'Planificateur de projet'!A$4=MEDIAN('Planificateur de projet'!A$4,'Planificateur de projet'!$C1,'Planificateur de projet'!$C1+'Planificateur de projet'!$D1-1)</definedName>
     <definedName name="PériodeDansRéel">'Planificateur de projet'!A$4=MEDIAN('Planificateur de projet'!A$4,'Planificateur de projet'!$E1,'Planificateur de projet'!$E1+'Planificateur de projet'!$F1-1)</definedName>
     <definedName name="Plan">PériodeDansPlan*('Planificateur de projet'!$C1&gt;0)</definedName>
     <definedName name="PourcentageAccompli">PourcentageAccompliAuDelà*PériodeDansPlan</definedName>
     <definedName name="PourcentageAccompliAuDelà">('Planificateur de projet'!A$4=MEDIAN('Planificateur de projet'!A$4,'Planificateur de projet'!$E1,'Planificateur de projet'!$E1+'Planificateur de projet'!$F1)*('Planificateur de projet'!$E1&gt;0))*(('Planificateur de projet'!A$4&lt;(INT('Planificateur de projet'!$E1+'Planificateur de projet'!$F1*'Planificateur de projet'!$G1)))+('Planificateur de projet'!A$4='Planificateur de projet'!$E1))*('Planificateur de projet'!$G1&gt;0)</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Planificateur de projet'!$3:$4</definedName>
     <definedName name="Réel">(PériodeDansRéel*('Planificateur de projet'!$E1&gt;0))*PériodeDansPlan</definedName>
     <definedName name="RéelAuDelà">PériodeDansRéel*('Planificateur de projet'!$E1&gt;0)</definedName>
     <definedName name="TitreRégion..BO60">'Planificateur de projet'!$B$3:$B$4</definedName>
@@ -821,18 +821,18 @@
     <cellStyle name="En-têtes de période" xfId="3" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
     <cellStyle name="En-têtes de projet" xfId="4" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
     <cellStyle name="Étiquette" xfId="5" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="Explanatory Text" xfId="12" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="1" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="9" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="10" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="11" builtinId="19" customBuiltin="1"/>
     <cellStyle name="Légende de ce qui a été accompli" xfId="15" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
     <cellStyle name="Légende de ce qui a été accompli (au-delà du plan)" xfId="17" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="Légende du % accompli (au-delà du plan)" xfId="18" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Légende du plan" xfId="14" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
     <cellStyle name="Pourcentage accompli" xfId="6" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
-    <cellStyle name="Title" xfId="8" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Texte explicatif" xfId="12" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Titre" xfId="8" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Titre 1" xfId="1" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Titre 2" xfId="9" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Titre 3" xfId="10" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Titre 4" xfId="11" builtinId="19" customBuiltin="1"/>
     <cellStyle name="Valeur de la période" xfId="13" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
   </cellStyles>
   <dxfs count="9">
@@ -1214,20 +1214,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:XD55"/>
-  <sheetFormatPr defaultColWidth="3.25" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="3.25" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.58203125" customWidth="1"/>
+    <col min="1" max="1" width="2.625" customWidth="1"/>
     <col min="2" max="2" width="27.75" style="2" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.375" style="1" customWidth="1"/>
     <col min="5" max="5" width="12.5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.33203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18.375" style="1" customWidth="1"/>
     <col min="7" max="7" width="25.5" style="3" customWidth="1"/>
     <col min="8" max="27" width="3.25" style="1"/>
-    <col min="112" max="112" width="3.58203125" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="3.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:628" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="1.25">
+    <row r="1" spans="1:628" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A1" s="9"/>
       <c r="B1" s="13" t="s">
         <v>0</v>
@@ -1390,7 +1390,7 @@
       <c r="FB1" s="9"/>
       <c r="FC1" s="9"/>
     </row>
-    <row r="2" spans="1:628" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:628" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9"/>
       <c r="B2" s="15" t="s">
         <v>1</v>
@@ -1403,7 +1403,7 @@
         <v>7</v>
       </c>
       <c r="H2" s="17">
-        <v>48</v>
+        <v>80</v>
       </c>
       <c r="I2" s="8"/>
       <c r="J2" s="18"/>
@@ -2036,7 +2036,7 @@
       <c r="XC2" s="9"/>
       <c r="XD2" s="9"/>
     </row>
-    <row r="3" spans="1:628" s="4" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:628" s="4" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11"/>
       <c r="B3" s="39" t="s">
         <v>2</v>
@@ -2680,7 +2680,7 @@
       <c r="XC3" s="11"/>
       <c r="XD3" s="11"/>
     </row>
-    <row r="4" spans="1:628" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:628" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="9"/>
       <c r="B4" s="40"/>
       <c r="C4" s="42"/>
@@ -3520,7 +3520,7 @@
       <c r="XC4" s="9"/>
       <c r="XD4" s="9"/>
     </row>
-    <row r="6" spans="1:628" s="9" customFormat="1" ht="17" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:628" s="9" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>31</v>
       </c>
@@ -3560,7 +3560,7 @@
       <c r="Z6" s="8"/>
       <c r="AA6" s="8"/>
     </row>
-    <row r="7" spans="1:628" s="9" customFormat="1" ht="17" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:628" s="9" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>32</v>
       </c>
@@ -3600,7 +3600,7 @@
       <c r="Z7" s="8"/>
       <c r="AA7" s="8"/>
     </row>
-    <row r="8" spans="1:628" s="9" customFormat="1" ht="17" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:628" s="9" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>15</v>
       </c>
@@ -3640,7 +3640,7 @@
       <c r="Z8" s="8"/>
       <c r="AA8" s="8"/>
     </row>
-    <row r="9" spans="1:628" s="9" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:628" s="9" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>30</v>
       </c>
@@ -3680,7 +3680,7 @@
       <c r="Z9" s="8"/>
       <c r="AA9" s="8"/>
     </row>
-    <row r="10" spans="1:628" s="9" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:628" s="9" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="5" t="s">
         <v>16</v>
       </c>
@@ -3720,7 +3720,7 @@
       <c r="Z10" s="8"/>
       <c r="AA10" s="8"/>
     </row>
-    <row r="11" spans="1:628" s="10" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:628" s="10" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9"/>
       <c r="B11" s="5" t="s">
         <v>17</v>
@@ -4362,7 +4362,7 @@
       <c r="XC11" s="9"/>
       <c r="XD11" s="9"/>
     </row>
-    <row r="12" spans="1:628" s="9" customFormat="1" ht="17" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:628" s="9" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
       <c r="B12" s="5" t="s">
         <v>18</v>
       </c>
@@ -4402,7 +4402,7 @@
       <c r="Z12" s="8"/>
       <c r="AA12" s="8"/>
     </row>
-    <row r="13" spans="1:628" ht="34" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:628" ht="34.5" x14ac:dyDescent="0.3">
       <c r="A13" s="9"/>
       <c r="B13" s="5" t="s">
         <v>34</v>
@@ -5044,7 +5044,7 @@
       <c r="XC13" s="9"/>
       <c r="XD13" s="9"/>
     </row>
-    <row r="14" spans="1:628" ht="31.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:628" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="9"/>
       <c r="B14" s="5" t="s">
         <v>35</v>
@@ -5686,7 +5686,7 @@
       <c r="XC14" s="9"/>
       <c r="XD14" s="9"/>
     </row>
-    <row r="15" spans="1:628" ht="34" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:628" ht="34.5" x14ac:dyDescent="0.3">
       <c r="A15" s="9"/>
       <c r="B15" s="5" t="s">
         <v>19</v>
@@ -6328,7 +6328,7 @@
       <c r="XC15" s="9"/>
       <c r="XD15" s="9"/>
     </row>
-    <row r="16" spans="1:628" s="9" customFormat="1" ht="17" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:628" s="9" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>20</v>
       </c>
@@ -6368,7 +6368,7 @@
       <c r="Z16" s="8"/>
       <c r="AA16" s="8"/>
     </row>
-    <row r="17" spans="1:628" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:628" s="10" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A17" s="9"/>
       <c r="B17" s="5" t="s">
         <v>21</v>
@@ -7010,7 +7010,7 @@
       <c r="XC17" s="9"/>
       <c r="XD17" s="9"/>
     </row>
-    <row r="18" spans="1:628" s="9" customFormat="1" ht="17" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:628" s="9" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
       <c r="B18" s="5" t="s">
         <v>65</v>
       </c>
@@ -7050,7 +7050,7 @@
       <c r="Z18" s="8"/>
       <c r="AA18" s="8"/>
     </row>
-    <row r="19" spans="1:628" ht="17" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:628" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A19" s="9"/>
       <c r="B19" s="5" t="s">
         <v>22</v>
@@ -7065,10 +7065,10 @@
         <v>48</v>
       </c>
       <c r="F19" s="6">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G19" s="7">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="H19" s="8"/>
       <c r="I19" s="8"/>
@@ -7692,7 +7692,7 @@
       <c r="XC19" s="9"/>
       <c r="XD19" s="9"/>
     </row>
-    <row r="20" spans="1:628" ht="34" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:628" ht="34.5" x14ac:dyDescent="0.3">
       <c r="A20" s="9"/>
       <c r="B20" s="5" t="s">
         <v>23</v>
@@ -7710,7 +7710,7 @@
         <v>9</v>
       </c>
       <c r="G20" s="7">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
@@ -8334,7 +8334,7 @@
       <c r="XC20" s="9"/>
       <c r="XD20" s="9"/>
     </row>
-    <row r="21" spans="1:628" ht="17" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:628" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A21" s="9"/>
       <c r="B21" s="5" t="s">
         <v>24</v>
@@ -8974,7 +8974,7 @@
       <c r="XC21" s="9"/>
       <c r="XD21" s="9"/>
     </row>
-    <row r="22" spans="1:628" s="9" customFormat="1" ht="34" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:628" s="9" customFormat="1" ht="34.5" x14ac:dyDescent="0.3">
       <c r="B22" s="5" t="s">
         <v>25</v>
       </c>
@@ -9012,7 +9012,7 @@
       <c r="Z22" s="8"/>
       <c r="AA22" s="8"/>
     </row>
-    <row r="23" spans="1:628" s="10" customFormat="1" ht="34" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:628" s="10" customFormat="1" ht="34.5" x14ac:dyDescent="0.3">
       <c r="A23" s="9"/>
       <c r="B23" s="5" t="s">
         <v>26</v>
@@ -9652,7 +9652,7 @@
       <c r="XC23" s="9"/>
       <c r="XD23" s="9"/>
     </row>
-    <row r="24" spans="1:628" s="9" customFormat="1" ht="34" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:628" s="9" customFormat="1" ht="34.5" x14ac:dyDescent="0.3">
       <c r="B24" s="5" t="s">
         <v>27</v>
       </c>
@@ -9690,7 +9690,7 @@
       <c r="Z24" s="8"/>
       <c r="AA24" s="8"/>
     </row>
-    <row r="25" spans="1:628" ht="54.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:628" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="9"/>
       <c r="B25" s="5" t="s">
         <v>28</v>
@@ -10330,7 +10330,7 @@
       <c r="XC25" s="9"/>
       <c r="XD25" s="9"/>
     </row>
-    <row r="26" spans="1:628" ht="48" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:628" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="9"/>
       <c r="B26" s="5" t="s">
         <v>29</v>
@@ -10970,7 +10970,7 @@
       <c r="XC26" s="9"/>
       <c r="XD26" s="9"/>
     </row>
-    <row r="27" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9"/>
       <c r="B27" s="5" t="s">
         <v>33</v>
@@ -11612,7 +11612,7 @@
       <c r="XC27" s="9"/>
       <c r="XD27" s="9"/>
     </row>
-    <row r="28" spans="1:628" s="9" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:628" s="9" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H28" s="8"/>
       <c r="I28" s="8"/>
       <c r="J28" s="8"/>
@@ -11634,7 +11634,7 @@
       <c r="Z28" s="8"/>
       <c r="AA28" s="8"/>
     </row>
-    <row r="29" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9"/>
       <c r="B29" s="26"/>
       <c r="C29" s="8"/>
@@ -12264,7 +12264,7 @@
       <c r="XC29" s="9"/>
       <c r="XD29" s="9"/>
     </row>
-    <row r="30" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="9"/>
       <c r="B30" s="26"/>
       <c r="C30" s="8"/>
@@ -12894,7 +12894,7 @@
       <c r="XC30" s="9"/>
       <c r="XD30" s="9"/>
     </row>
-    <row r="31" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="9"/>
       <c r="B31" s="26"/>
       <c r="C31" s="8"/>
@@ -13524,7 +13524,7 @@
       <c r="XC31" s="9"/>
       <c r="XD31" s="9"/>
     </row>
-    <row r="32" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="9"/>
       <c r="B32" s="26"/>
       <c r="C32" s="8"/>
@@ -14154,7 +14154,7 @@
       <c r="XC32" s="9"/>
       <c r="XD32" s="9"/>
     </row>
-    <row r="33" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="9"/>
       <c r="B33" s="26"/>
       <c r="C33" s="8"/>
@@ -14784,7 +14784,7 @@
       <c r="XC33" s="9"/>
       <c r="XD33" s="9"/>
     </row>
-    <row r="34" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="9"/>
       <c r="B34" s="26"/>
       <c r="C34" s="8"/>
@@ -15414,7 +15414,7 @@
       <c r="XC34" s="9"/>
       <c r="XD34" s="9"/>
     </row>
-    <row r="35" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="9"/>
       <c r="B35" s="26"/>
       <c r="C35" s="8"/>
@@ -16044,7 +16044,7 @@
       <c r="XC35" s="9"/>
       <c r="XD35" s="9"/>
     </row>
-    <row r="36" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9"/>
       <c r="B36" s="26"/>
       <c r="C36" s="8"/>
@@ -16674,7 +16674,7 @@
       <c r="XC36" s="9"/>
       <c r="XD36" s="9"/>
     </row>
-    <row r="37" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="9"/>
       <c r="B37" s="26"/>
       <c r="C37" s="8"/>
@@ -17304,7 +17304,7 @@
       <c r="XC37" s="9"/>
       <c r="XD37" s="9"/>
     </row>
-    <row r="38" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="9"/>
       <c r="B38" s="26"/>
       <c r="C38" s="8"/>
@@ -17934,7 +17934,7 @@
       <c r="XC38" s="9"/>
       <c r="XD38" s="9"/>
     </row>
-    <row r="39" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="9"/>
       <c r="B39" s="26"/>
       <c r="C39" s="8"/>
@@ -18564,7 +18564,7 @@
       <c r="XC39" s="9"/>
       <c r="XD39" s="9"/>
     </row>
-    <row r="40" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="9"/>
       <c r="B40" s="26"/>
       <c r="C40" s="8"/>
@@ -19194,7 +19194,7 @@
       <c r="XC40" s="9"/>
       <c r="XD40" s="9"/>
     </row>
-    <row r="41" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="9"/>
       <c r="B41" s="26"/>
       <c r="C41" s="8"/>
@@ -19824,7 +19824,7 @@
       <c r="XC41" s="9"/>
       <c r="XD41" s="9"/>
     </row>
-    <row r="42" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="9"/>
       <c r="B42" s="26"/>
       <c r="C42" s="8"/>
@@ -20454,7 +20454,7 @@
       <c r="XC42" s="9"/>
       <c r="XD42" s="9"/>
     </row>
-    <row r="43" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="9"/>
       <c r="B43" s="26"/>
       <c r="C43" s="8"/>
@@ -21084,7 +21084,7 @@
       <c r="XC43" s="9"/>
       <c r="XD43" s="9"/>
     </row>
-    <row r="44" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="9"/>
       <c r="B44" s="26"/>
       <c r="C44" s="8"/>
@@ -21714,7 +21714,7 @@
       <c r="XC44" s="9"/>
       <c r="XD44" s="9"/>
     </row>
-    <row r="45" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="9"/>
       <c r="B45" s="26"/>
       <c r="C45" s="8"/>
@@ -21875,7 +21875,7 @@
       <c r="FB45" s="9"/>
       <c r="FC45" s="9"/>
     </row>
-    <row r="46" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="9"/>
       <c r="B46" s="26"/>
       <c r="C46" s="8"/>
@@ -22036,7 +22036,7 @@
       <c r="FB46" s="9"/>
       <c r="FC46" s="9"/>
     </row>
-    <row r="47" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9"/>
       <c r="B47" s="26"/>
       <c r="C47" s="8"/>
@@ -22197,7 +22197,7 @@
       <c r="FB47" s="9"/>
       <c r="FC47" s="9"/>
     </row>
-    <row r="48" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="9"/>
       <c r="B48" s="26"/>
       <c r="C48" s="8"/>
@@ -22358,7 +22358,7 @@
       <c r="FB48" s="9"/>
       <c r="FC48" s="9"/>
     </row>
-    <row r="49" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="9"/>
       <c r="B49" s="26"/>
       <c r="C49" s="8"/>
@@ -22519,7 +22519,7 @@
       <c r="FB49" s="9"/>
       <c r="FC49" s="9"/>
     </row>
-    <row r="50" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="9"/>
       <c r="B50" s="26"/>
       <c r="C50" s="8"/>
@@ -22680,7 +22680,7 @@
       <c r="FB50" s="9"/>
       <c r="FC50" s="9"/>
     </row>
-    <row r="51" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="9"/>
       <c r="B51" s="26"/>
       <c r="C51" s="8"/>
@@ -22841,7 +22841,7 @@
       <c r="FB51" s="9"/>
       <c r="FC51" s="9"/>
     </row>
-    <row r="52" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9"/>
       <c r="B52" s="26"/>
       <c r="C52" s="8"/>
@@ -23002,7 +23002,7 @@
       <c r="FB52" s="9"/>
       <c r="FC52" s="9"/>
     </row>
-    <row r="53" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="9"/>
       <c r="B53" s="26"/>
       <c r="C53" s="8"/>
@@ -23163,7 +23163,7 @@
       <c r="FB53" s="9"/>
       <c r="FC53" s="9"/>
     </row>
-    <row r="54" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="9"/>
       <c r="B54" s="26"/>
       <c r="C54" s="8"/>
@@ -23324,7 +23324,7 @@
       <c r="FB54" s="9"/>
       <c r="FC54" s="9"/>
     </row>
-    <row r="55" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="9"/>
       <c r="B55" s="26"/>
       <c r="C55" s="8"/>
@@ -23567,22 +23567,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E19089D2-0F21-4ACE-A307-C157013F582B}">
   <dimension ref="A2:D43"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.58203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="2.75" style="28" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="83.75" style="30" customWidth="1"/>
     <col min="5" max="5" width="40.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C2" s="35"/>
       <c r="D2" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="31" t="s">
         <v>36</v>
       </c>
@@ -23596,7 +23596,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C5" s="29" t="s">
         <v>45</v>
       </c>
@@ -23604,7 +23604,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="31" t="s">
         <v>37</v>
       </c>
@@ -23618,7 +23618,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C8" s="29" t="s">
         <v>45</v>
       </c>
@@ -23626,7 +23626,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="31" t="s">
         <v>38</v>
       </c>
@@ -23640,7 +23640,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="31" t="s">
         <v>39</v>
       </c>
@@ -23654,7 +23654,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C13" s="29" t="s">
         <v>45</v>
       </c>
@@ -23662,12 +23662,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D14" s="34" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="31" t="s">
         <v>36</v>
       </c>
@@ -23681,7 +23681,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="31" t="s">
         <v>37</v>
       </c>
@@ -23695,7 +23695,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C19" s="29" t="s">
         <v>55</v>
       </c>
@@ -23703,12 +23703,12 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D20" s="34" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="31" t="s">
         <v>38</v>
       </c>
@@ -23722,17 +23722,17 @@
         <v>57</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D23" s="30" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D24" s="34" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="31" t="s">
         <v>36</v>
       </c>
@@ -23746,7 +23746,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C27" s="29">
         <v>4</v>
       </c>
@@ -23754,7 +23754,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="31" t="s">
         <v>37</v>
       </c>
@@ -23768,7 +23768,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C30" s="28" t="s">
         <v>45</v>
       </c>
@@ -23776,7 +23776,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="31" t="s">
         <v>38</v>
       </c>
@@ -23790,7 +23790,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C33" s="29" t="s">
         <v>45</v>
       </c>
@@ -23798,12 +23798,12 @@
         <v>63</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D34" s="33" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="31" t="s">
         <v>36</v>
       </c>
@@ -23817,7 +23817,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="31" t="s">
         <v>37</v>
       </c>
@@ -23831,7 +23831,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C39" s="28" t="s">
         <v>45</v>
       </c>
@@ -23839,7 +23839,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C40" s="28" t="s">
         <v>46</v>
       </c>
@@ -23847,7 +23847,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="31" t="s">
         <v>38</v>
       </c>
@@ -23861,7 +23861,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C43" s="28" t="s">
         <v>46</v>
       </c>
@@ -24096,20 +24096,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="b00ac6d6-80cd-413d-830d-913bbb25803f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="b00ac6d6-80cd-413d-830d-913bbb25803f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -24132,14 +24132,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73E1A9BE-BAF3-41A8-A0B4-1FE716ABEFE3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93C7558B-A91F-4A35-B94E-E9BF71A53151}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -24154,4 +24146,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73E1A9BE-BAF3-41A8-A0B4-1FE716ABEFE3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Show warranty days left and format purchase date
Add warranty calculation and display improvements: import datetime utilities; add days_left(purchase_date, warranty_months) helper to compute remaining warranty days; replace hardcoded "12 days left" badge with the computed value and format purchase_date as DD-MM-YYYY (showing "None" when missing). Binary assets (.xlsx) and compiled .pyc files were also updated.
</commit_message>
<xml_diff>
--- a/Documentations/Planning-Journal_de_travail-TPI-Jimmy.xlsx
+++ b/Documentations/Planning-Journal_de_travail-TPI-Jimmy.xlsx
@@ -3,22 +3,22 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{324D871E-12D2-4654-B26A-53DCCB56C5A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0433E41-AAFF-41BC-934E-5FEA21CB5EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planificateur de projet" sheetId="1" r:id="rId1"/>
     <sheet name="Journal de travail" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Planificateur de projet'!$3:$4</definedName>
     <definedName name="période_sélectionnée">'Planificateur de projet'!$H$2</definedName>
     <definedName name="PériodeDansPlan">'Planificateur de projet'!A$4=MEDIAN('Planificateur de projet'!A$4,'Planificateur de projet'!$C1,'Planificateur de projet'!$C1+'Planificateur de projet'!$D1-1)</definedName>
     <definedName name="PériodeDansRéel">'Planificateur de projet'!A$4=MEDIAN('Planificateur de projet'!A$4,'Planificateur de projet'!$E1,'Planificateur de projet'!$E1+'Planificateur de projet'!$F1-1)</definedName>
     <definedName name="Plan">PériodeDansPlan*('Planificateur de projet'!$C1&gt;0)</definedName>
     <definedName name="PourcentageAccompli">PourcentageAccompliAuDelà*PériodeDansPlan</definedName>
     <definedName name="PourcentageAccompliAuDelà">('Planificateur de projet'!A$4=MEDIAN('Planificateur de projet'!A$4,'Planificateur de projet'!$E1,'Planificateur de projet'!$E1+'Planificateur de projet'!$F1)*('Planificateur de projet'!$E1&gt;0))*(('Planificateur de projet'!A$4&lt;(INT('Planificateur de projet'!$E1+'Planificateur de projet'!$F1*'Planificateur de projet'!$G1)))+('Planificateur de projet'!A$4='Planificateur de projet'!$E1))*('Planificateur de projet'!$G1&gt;0)</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Planificateur de projet'!$3:$4</definedName>
     <definedName name="Réel">(PériodeDansRéel*('Planificateur de projet'!$E1&gt;0))*PériodeDansPlan</definedName>
     <definedName name="RéelAuDelà">PériodeDansRéel*('Planificateur de projet'!$E1&gt;0)</definedName>
     <definedName name="TitreRégion..BO60">'Planificateur de projet'!$B$3:$B$4</definedName>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="75">
   <si>
     <t>Planificateur de projet</t>
   </si>
@@ -331,6 +331,15 @@
   </si>
   <si>
     <t>Recherche sur les meilleurs frameworks OCR, meilleur base de donné plus complete</t>
+  </si>
+  <si>
+    <t>Migration de easyocr vers doctr</t>
+  </si>
+  <si>
+    <t>Implémentation de doctr dans le main.py</t>
+  </si>
+  <si>
+    <t>Problème avec streamlit cloud. Je n'arrive pas a faire fonctionner l'application dans le cloud.</t>
   </si>
 </sst>
 </file>
@@ -821,18 +830,18 @@
     <cellStyle name="En-têtes de période" xfId="3" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
     <cellStyle name="En-têtes de projet" xfId="4" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
     <cellStyle name="Étiquette" xfId="5" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="Explanatory Text" xfId="12" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="1" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="9" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="10" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="11" builtinId="19" customBuiltin="1"/>
     <cellStyle name="Légende de ce qui a été accompli" xfId="15" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
     <cellStyle name="Légende de ce qui a été accompli (au-delà du plan)" xfId="17" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="Légende du % accompli (au-delà du plan)" xfId="18" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Légende du plan" xfId="14" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
     <cellStyle name="Pourcentage accompli" xfId="6" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
-    <cellStyle name="Texte explicatif" xfId="12" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Titre" xfId="8" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Titre 1" xfId="1" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Titre 2" xfId="9" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Titre 3" xfId="10" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Titre 4" xfId="11" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="8" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Valeur de la période" xfId="13" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
   </cellStyles>
   <dxfs count="9">
@@ -1214,20 +1223,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:XD55"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="3.25" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="3.25" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="2.625" customWidth="1"/>
+    <col min="1" max="1" width="2.58203125" customWidth="1"/>
     <col min="2" max="2" width="27.75" style="2" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15.375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" style="1" customWidth="1"/>
     <col min="5" max="5" width="12.5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18.33203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="25.5" style="3" customWidth="1"/>
     <col min="8" max="27" width="3.25" style="1"/>
-    <col min="112" max="112" width="3.625" bestFit="1" customWidth="1"/>
+    <col min="112" max="112" width="3.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:628" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.85">
+    <row r="1" spans="1:628" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="1.25">
       <c r="A1" s="9"/>
       <c r="B1" s="13" t="s">
         <v>0</v>
@@ -1390,7 +1399,7 @@
       <c r="FB1" s="9"/>
       <c r="FC1" s="9"/>
     </row>
-    <row r="2" spans="1:628" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:628" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9"/>
       <c r="B2" s="15" t="s">
         <v>1</v>
@@ -2036,7 +2045,7 @@
       <c r="XC2" s="9"/>
       <c r="XD2" s="9"/>
     </row>
-    <row r="3" spans="1:628" s="4" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:628" s="4" customFormat="1" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A3" s="11"/>
       <c r="B3" s="39" t="s">
         <v>2</v>
@@ -2680,7 +2689,7 @@
       <c r="XC3" s="11"/>
       <c r="XD3" s="11"/>
     </row>
-    <row r="4" spans="1:628" ht="15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:628" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A4" s="9"/>
       <c r="B4" s="40"/>
       <c r="C4" s="42"/>
@@ -3520,7 +3529,7 @@
       <c r="XC4" s="9"/>
       <c r="XD4" s="9"/>
     </row>
-    <row r="6" spans="1:628" s="9" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:628" s="9" customFormat="1" ht="17" x14ac:dyDescent="0.4">
       <c r="B6" s="5" t="s">
         <v>31</v>
       </c>
@@ -3560,7 +3569,7 @@
       <c r="Z6" s="8"/>
       <c r="AA6" s="8"/>
     </row>
-    <row r="7" spans="1:628" s="9" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:628" s="9" customFormat="1" ht="17" x14ac:dyDescent="0.4">
       <c r="B7" s="5" t="s">
         <v>32</v>
       </c>
@@ -3600,7 +3609,7 @@
       <c r="Z7" s="8"/>
       <c r="AA7" s="8"/>
     </row>
-    <row r="8" spans="1:628" s="9" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:628" s="9" customFormat="1" ht="17" x14ac:dyDescent="0.4">
       <c r="B8" s="5" t="s">
         <v>15</v>
       </c>
@@ -3640,7 +3649,7 @@
       <c r="Z8" s="8"/>
       <c r="AA8" s="8"/>
     </row>
-    <row r="9" spans="1:628" s="9" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:628" s="9" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B9" s="5" t="s">
         <v>30</v>
       </c>
@@ -3680,7 +3689,7 @@
       <c r="Z9" s="8"/>
       <c r="AA9" s="8"/>
     </row>
-    <row r="10" spans="1:628" s="9" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:628" s="9" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B10" s="5" t="s">
         <v>16</v>
       </c>
@@ -3720,7 +3729,7 @@
       <c r="Z10" s="8"/>
       <c r="AA10" s="8"/>
     </row>
-    <row r="11" spans="1:628" s="10" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:628" s="10" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="9"/>
       <c r="B11" s="5" t="s">
         <v>17</v>
@@ -4362,7 +4371,7 @@
       <c r="XC11" s="9"/>
       <c r="XD11" s="9"/>
     </row>
-    <row r="12" spans="1:628" s="9" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:628" s="9" customFormat="1" ht="17" x14ac:dyDescent="0.4">
       <c r="B12" s="5" t="s">
         <v>18</v>
       </c>
@@ -4402,7 +4411,7 @@
       <c r="Z12" s="8"/>
       <c r="AA12" s="8"/>
     </row>
-    <row r="13" spans="1:628" ht="34.5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:628" ht="34" x14ac:dyDescent="0.4">
       <c r="A13" s="9"/>
       <c r="B13" s="5" t="s">
         <v>34</v>
@@ -5044,7 +5053,7 @@
       <c r="XC13" s="9"/>
       <c r="XD13" s="9"/>
     </row>
-    <row r="14" spans="1:628" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:628" ht="31.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="9"/>
       <c r="B14" s="5" t="s">
         <v>35</v>
@@ -5686,7 +5695,7 @@
       <c r="XC14" s="9"/>
       <c r="XD14" s="9"/>
     </row>
-    <row r="15" spans="1:628" ht="34.5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:628" ht="34" x14ac:dyDescent="0.4">
       <c r="A15" s="9"/>
       <c r="B15" s="5" t="s">
         <v>19</v>
@@ -6328,7 +6337,7 @@
       <c r="XC15" s="9"/>
       <c r="XD15" s="9"/>
     </row>
-    <row r="16" spans="1:628" s="9" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:628" s="9" customFormat="1" ht="17" x14ac:dyDescent="0.4">
       <c r="B16" s="5" t="s">
         <v>20</v>
       </c>
@@ -6368,7 +6377,7 @@
       <c r="Z16" s="8"/>
       <c r="AA16" s="8"/>
     </row>
-    <row r="17" spans="1:628" s="10" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:628" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.4">
       <c r="A17" s="9"/>
       <c r="B17" s="5" t="s">
         <v>21</v>
@@ -7010,7 +7019,7 @@
       <c r="XC17" s="9"/>
       <c r="XD17" s="9"/>
     </row>
-    <row r="18" spans="1:628" s="9" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:628" s="9" customFormat="1" ht="17" x14ac:dyDescent="0.4">
       <c r="B18" s="5" t="s">
         <v>65</v>
       </c>
@@ -7050,7 +7059,7 @@
       <c r="Z18" s="8"/>
       <c r="AA18" s="8"/>
     </row>
-    <row r="19" spans="1:628" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:628" ht="17" x14ac:dyDescent="0.4">
       <c r="A19" s="9"/>
       <c r="B19" s="5" t="s">
         <v>22</v>
@@ -7692,7 +7701,7 @@
       <c r="XC19" s="9"/>
       <c r="XD19" s="9"/>
     </row>
-    <row r="20" spans="1:628" ht="34.5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:628" ht="34" x14ac:dyDescent="0.4">
       <c r="A20" s="9"/>
       <c r="B20" s="5" t="s">
         <v>23</v>
@@ -8334,7 +8343,7 @@
       <c r="XC20" s="9"/>
       <c r="XD20" s="9"/>
     </row>
-    <row r="21" spans="1:628" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:628" ht="17" x14ac:dyDescent="0.4">
       <c r="A21" s="9"/>
       <c r="B21" s="5" t="s">
         <v>24</v>
@@ -8974,7 +8983,7 @@
       <c r="XC21" s="9"/>
       <c r="XD21" s="9"/>
     </row>
-    <row r="22" spans="1:628" s="9" customFormat="1" ht="34.5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:628" s="9" customFormat="1" ht="34" x14ac:dyDescent="0.4">
       <c r="B22" s="5" t="s">
         <v>25</v>
       </c>
@@ -9012,7 +9021,7 @@
       <c r="Z22" s="8"/>
       <c r="AA22" s="8"/>
     </row>
-    <row r="23" spans="1:628" s="10" customFormat="1" ht="34.5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:628" s="10" customFormat="1" ht="34" x14ac:dyDescent="0.4">
       <c r="A23" s="9"/>
       <c r="B23" s="5" t="s">
         <v>26</v>
@@ -9023,7 +9032,9 @@
       <c r="D23" s="6">
         <v>4</v>
       </c>
-      <c r="E23" s="6"/>
+      <c r="E23" s="6">
+        <v>0</v>
+      </c>
       <c r="F23" s="6">
         <v>0</v>
       </c>
@@ -9652,7 +9663,7 @@
       <c r="XC23" s="9"/>
       <c r="XD23" s="9"/>
     </row>
-    <row r="24" spans="1:628" s="9" customFormat="1" ht="34.5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:628" s="9" customFormat="1" ht="34" x14ac:dyDescent="0.4">
       <c r="B24" s="5" t="s">
         <v>27</v>
       </c>
@@ -9662,12 +9673,14 @@
       <c r="D24" s="6">
         <v>3</v>
       </c>
-      <c r="E24" s="6"/>
+      <c r="E24" s="6">
+        <v>64</v>
+      </c>
       <c r="F24" s="6">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G24" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H24" s="8"/>
       <c r="I24" s="8"/>
@@ -9690,7 +9703,7 @@
       <c r="Z24" s="8"/>
       <c r="AA24" s="8"/>
     </row>
-    <row r="25" spans="1:628" ht="54.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:628" ht="54.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="9"/>
       <c r="B25" s="5" t="s">
         <v>28</v>
@@ -10330,7 +10343,7 @@
       <c r="XC25" s="9"/>
       <c r="XD25" s="9"/>
     </row>
-    <row r="26" spans="1:628" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:628" ht="48" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="9"/>
       <c r="B26" s="5" t="s">
         <v>29</v>
@@ -10970,7 +10983,7 @@
       <c r="XC26" s="9"/>
       <c r="XD26" s="9"/>
     </row>
-    <row r="27" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="9"/>
       <c r="B27" s="5" t="s">
         <v>33</v>
@@ -11612,7 +11625,7 @@
       <c r="XC27" s="9"/>
       <c r="XD27" s="9"/>
     </row>
-    <row r="28" spans="1:628" s="9" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:628" s="9" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="H28" s="8"/>
       <c r="I28" s="8"/>
       <c r="J28" s="8"/>
@@ -11634,7 +11647,7 @@
       <c r="Z28" s="8"/>
       <c r="AA28" s="8"/>
     </row>
-    <row r="29" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="9"/>
       <c r="B29" s="26"/>
       <c r="C29" s="8"/>
@@ -12264,7 +12277,7 @@
       <c r="XC29" s="9"/>
       <c r="XD29" s="9"/>
     </row>
-    <row r="30" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="9"/>
       <c r="B30" s="26"/>
       <c r="C30" s="8"/>
@@ -12894,7 +12907,7 @@
       <c r="XC30" s="9"/>
       <c r="XD30" s="9"/>
     </row>
-    <row r="31" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="9"/>
       <c r="B31" s="26"/>
       <c r="C31" s="8"/>
@@ -13524,7 +13537,7 @@
       <c r="XC31" s="9"/>
       <c r="XD31" s="9"/>
     </row>
-    <row r="32" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="9"/>
       <c r="B32" s="26"/>
       <c r="C32" s="8"/>
@@ -14154,7 +14167,7 @@
       <c r="XC32" s="9"/>
       <c r="XD32" s="9"/>
     </row>
-    <row r="33" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="9"/>
       <c r="B33" s="26"/>
       <c r="C33" s="8"/>
@@ -14784,7 +14797,7 @@
       <c r="XC33" s="9"/>
       <c r="XD33" s="9"/>
     </row>
-    <row r="34" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="9"/>
       <c r="B34" s="26"/>
       <c r="C34" s="8"/>
@@ -15414,7 +15427,7 @@
       <c r="XC34" s="9"/>
       <c r="XD34" s="9"/>
     </row>
-    <row r="35" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="9"/>
       <c r="B35" s="26"/>
       <c r="C35" s="8"/>
@@ -16044,7 +16057,7 @@
       <c r="XC35" s="9"/>
       <c r="XD35" s="9"/>
     </row>
-    <row r="36" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="9"/>
       <c r="B36" s="26"/>
       <c r="C36" s="8"/>
@@ -16674,7 +16687,7 @@
       <c r="XC36" s="9"/>
       <c r="XD36" s="9"/>
     </row>
-    <row r="37" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="9"/>
       <c r="B37" s="26"/>
       <c r="C37" s="8"/>
@@ -17304,7 +17317,7 @@
       <c r="XC37" s="9"/>
       <c r="XD37" s="9"/>
     </row>
-    <row r="38" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="9"/>
       <c r="B38" s="26"/>
       <c r="C38" s="8"/>
@@ -17934,7 +17947,7 @@
       <c r="XC38" s="9"/>
       <c r="XD38" s="9"/>
     </row>
-    <row r="39" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:628" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A39" s="9"/>
       <c r="B39" s="26"/>
       <c r="C39" s="8"/>
@@ -18564,7 +18577,7 @@
       <c r="XC39" s="9"/>
       <c r="XD39" s="9"/>
     </row>
-    <row r="40" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A40" s="9"/>
       <c r="B40" s="26"/>
       <c r="C40" s="8"/>
@@ -19194,7 +19207,7 @@
       <c r="XC40" s="9"/>
       <c r="XD40" s="9"/>
     </row>
-    <row r="41" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A41" s="9"/>
       <c r="B41" s="26"/>
       <c r="C41" s="8"/>
@@ -19824,7 +19837,7 @@
       <c r="XC41" s="9"/>
       <c r="XD41" s="9"/>
     </row>
-    <row r="42" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A42" s="9"/>
       <c r="B42" s="26"/>
       <c r="C42" s="8"/>
@@ -20454,7 +20467,7 @@
       <c r="XC42" s="9"/>
       <c r="XD42" s="9"/>
     </row>
-    <row r="43" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A43" s="9"/>
       <c r="B43" s="26"/>
       <c r="C43" s="8"/>
@@ -21084,7 +21097,7 @@
       <c r="XC43" s="9"/>
       <c r="XD43" s="9"/>
     </row>
-    <row r="44" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A44" s="9"/>
       <c r="B44" s="26"/>
       <c r="C44" s="8"/>
@@ -21714,7 +21727,7 @@
       <c r="XC44" s="9"/>
       <c r="XD44" s="9"/>
     </row>
-    <row r="45" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A45" s="9"/>
       <c r="B45" s="26"/>
       <c r="C45" s="8"/>
@@ -21875,7 +21888,7 @@
       <c r="FB45" s="9"/>
       <c r="FC45" s="9"/>
     </row>
-    <row r="46" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A46" s="9"/>
       <c r="B46" s="26"/>
       <c r="C46" s="8"/>
@@ -22036,7 +22049,7 @@
       <c r="FB46" s="9"/>
       <c r="FC46" s="9"/>
     </row>
-    <row r="47" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A47" s="9"/>
       <c r="B47" s="26"/>
       <c r="C47" s="8"/>
@@ -22197,7 +22210,7 @@
       <c r="FB47" s="9"/>
       <c r="FC47" s="9"/>
     </row>
-    <row r="48" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:628" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A48" s="9"/>
       <c r="B48" s="26"/>
       <c r="C48" s="8"/>
@@ -22358,7 +22371,7 @@
       <c r="FB48" s="9"/>
       <c r="FC48" s="9"/>
     </row>
-    <row r="49" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A49" s="9"/>
       <c r="B49" s="26"/>
       <c r="C49" s="8"/>
@@ -22519,7 +22532,7 @@
       <c r="FB49" s="9"/>
       <c r="FC49" s="9"/>
     </row>
-    <row r="50" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A50" s="9"/>
       <c r="B50" s="26"/>
       <c r="C50" s="8"/>
@@ -22680,7 +22693,7 @@
       <c r="FB50" s="9"/>
       <c r="FC50" s="9"/>
     </row>
-    <row r="51" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A51" s="9"/>
       <c r="B51" s="26"/>
       <c r="C51" s="8"/>
@@ -22841,7 +22854,7 @@
       <c r="FB51" s="9"/>
       <c r="FC51" s="9"/>
     </row>
-    <row r="52" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A52" s="9"/>
       <c r="B52" s="26"/>
       <c r="C52" s="8"/>
@@ -23002,7 +23015,7 @@
       <c r="FB52" s="9"/>
       <c r="FC52" s="9"/>
     </row>
-    <row r="53" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A53" s="9"/>
       <c r="B53" s="26"/>
       <c r="C53" s="8"/>
@@ -23163,7 +23176,7 @@
       <c r="FB53" s="9"/>
       <c r="FC53" s="9"/>
     </row>
-    <row r="54" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A54" s="9"/>
       <c r="B54" s="26"/>
       <c r="C54" s="8"/>
@@ -23324,7 +23337,7 @@
       <c r="FB54" s="9"/>
       <c r="FC54" s="9"/>
     </row>
-    <row r="55" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:159" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A55" s="9"/>
       <c r="B55" s="26"/>
       <c r="C55" s="8"/>
@@ -23566,23 +23579,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E19089D2-0F21-4ACE-A307-C157013F582B}">
-  <dimension ref="A2:D43"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:D52"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.58203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="2.75" style="28" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="83.75" style="30" customWidth="1"/>
     <col min="5" max="5" width="40.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C2" s="35"/>
       <c r="D2" s="29" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="31" t="s">
         <v>36</v>
       </c>
@@ -23596,7 +23609,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C5" s="29" t="s">
         <v>45</v>
       </c>
@@ -23604,7 +23617,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="31" t="s">
         <v>37</v>
       </c>
@@ -23618,7 +23631,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C8" s="29" t="s">
         <v>45</v>
       </c>
@@ -23626,7 +23639,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="31" t="s">
         <v>38</v>
       </c>
@@ -23640,7 +23653,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="31" t="s">
         <v>39</v>
       </c>
@@ -23654,7 +23667,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C13" s="29" t="s">
         <v>45</v>
       </c>
@@ -23662,12 +23675,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D14" s="34" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="31" t="s">
         <v>36</v>
       </c>
@@ -23681,7 +23694,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="31" t="s">
         <v>37</v>
       </c>
@@ -23695,7 +23708,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C19" s="29" t="s">
         <v>55</v>
       </c>
@@ -23703,12 +23716,12 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D20" s="34" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="31" t="s">
         <v>38</v>
       </c>
@@ -23722,17 +23735,17 @@
         <v>57</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D23" s="30" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D24" s="34" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="31" t="s">
         <v>36</v>
       </c>
@@ -23746,7 +23759,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C27" s="29">
         <v>4</v>
       </c>
@@ -23754,7 +23767,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="31" t="s">
         <v>37</v>
       </c>
@@ -23768,7 +23781,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C30" s="28" t="s">
         <v>45</v>
       </c>
@@ -23776,7 +23789,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="31" t="s">
         <v>38</v>
       </c>
@@ -23790,7 +23803,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C33" s="29" t="s">
         <v>45</v>
       </c>
@@ -23798,12 +23811,12 @@
         <v>63</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D34" s="33" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="31" t="s">
         <v>36</v>
       </c>
@@ -23817,7 +23830,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="31" t="s">
         <v>37</v>
       </c>
@@ -23831,7 +23844,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C39" s="28" t="s">
         <v>45</v>
       </c>
@@ -23839,7 +23852,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C40" s="28" t="s">
         <v>46</v>
       </c>
@@ -23847,7 +23860,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="31" t="s">
         <v>38</v>
       </c>
@@ -23861,12 +23874,62 @@
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C43" s="28" t="s">
         <v>46</v>
       </c>
       <c r="D43" s="30" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="B45" s="32">
+        <v>46097</v>
+      </c>
+      <c r="C45" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="D45" s="30" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47" s="31" t="s">
+        <v>37</v>
+      </c>
+      <c r="B47" s="32">
+        <v>46098</v>
+      </c>
+      <c r="C47" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="D47" s="30" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C48" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="D48" s="30" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="B52" s="32">
+        <v>46100</v>
+      </c>
+      <c r="C52" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="D52" s="30" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -24096,20 +24159,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="b00ac6d6-80cd-413d-830d-913bbb25803f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="b00ac6d6-80cd-413d-830d-913bbb25803f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -24132,6 +24195,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73E1A9BE-BAF3-41A8-A0B4-1FE716ABEFE3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93C7558B-A91F-4A35-B94E-E9BF71A53151}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -24146,12 +24217,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73E1A9BE-BAF3-41A8-A0B4-1FE716ABEFE3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update documentation and planning workbook
Apply updates to project documentation and planning workbook. Modified Documentations/Documentation.docx and Documentations/Planning-Journal_de_travail-TPI-Jimmy.xlsx (binary files) to include the latest content/formatting changes; no source code affected.
</commit_message>
<xml_diff>
--- a/Documentations/Planning-Journal_de_travail-TPI-Jimmy.xlsx
+++ b/Documentations/Planning-Journal_de_travail-TPI-Jimmy.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0433E41-AAFF-41BC-934E-5FEA21CB5EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E8AC29-C174-4FDA-84B3-0BF8208D6AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="15200" windowHeight="21690" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planificateur de projet" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="77">
   <si>
     <t>Planificateur de projet</t>
   </si>
@@ -340,6 +340,12 @@
   </si>
   <si>
     <t>Problème avec streamlit cloud. Je n'arrive pas a faire fonctionner l'application dans le cloud.</t>
+  </si>
+  <si>
+    <t>Création du "module" login et bloquage des fonctionnalités si pas login</t>
+  </si>
+  <si>
+    <t>6p</t>
   </si>
 </sst>
 </file>
@@ -7033,7 +7039,7 @@
         <v>39</v>
       </c>
       <c r="F18" s="6">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G18" s="7">
         <v>1</v>
@@ -7074,7 +7080,7 @@
         <v>48</v>
       </c>
       <c r="F19" s="6">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="G19" s="7">
         <v>1</v>
@@ -9677,7 +9683,7 @@
         <v>64</v>
       </c>
       <c r="F24" s="6">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="G24" s="7">
         <v>1</v>
@@ -9714,7 +9720,9 @@
       <c r="D25" s="6">
         <v>7</v>
       </c>
-      <c r="E25" s="6"/>
+      <c r="E25" s="6">
+        <v>0</v>
+      </c>
       <c r="F25" s="6">
         <v>0</v>
       </c>
@@ -10354,12 +10362,14 @@
       <c r="D26" s="6">
         <v>10</v>
       </c>
-      <c r="E26" s="6"/>
+      <c r="E26" s="6">
+        <v>91</v>
+      </c>
       <c r="F26" s="6">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G26" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H26" s="8"/>
       <c r="I26" s="8"/>
@@ -10998,10 +11008,10 @@
         <v>1</v>
       </c>
       <c r="F27" s="6">
-        <v>64</v>
+        <v>105</v>
       </c>
       <c r="G27" s="7">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H27" s="8"/>
       <c r="I27" s="8"/>
@@ -23579,7 +23589,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E19089D2-0F21-4ACE-A307-C157013F582B}">
-  <dimension ref="A2:D52"/>
+  <dimension ref="A2:D56"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.58203125" bestFit="1" customWidth="1"/>
@@ -23918,18 +23928,60 @@
         <v>69</v>
       </c>
     </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="B50" s="32">
+        <v>46100</v>
+      </c>
+      <c r="C50" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="D50" s="30" t="s">
+        <v>74</v>
+      </c>
+    </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="B52" s="32">
+        <v>46104</v>
+      </c>
+      <c r="C52" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="D52" s="30" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" s="31" t="s">
+        <v>37</v>
+      </c>
+      <c r="B54" s="32">
+        <v>46105</v>
+      </c>
+      <c r="C54" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="D54" s="30" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="B52" s="32">
-        <v>46100</v>
-      </c>
-      <c r="C52" s="28" t="s">
+      <c r="B56" s="32">
+        <v>46079</v>
+      </c>
+      <c r="C56" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="D52" s="30" t="s">
-        <v>74</v>
+      <c r="D56" s="33" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -24159,20 +24211,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="b00ac6d6-80cd-413d-830d-913bbb25803f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="b00ac6d6-80cd-413d-830d-913bbb25803f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -24195,14 +24247,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73E1A9BE-BAF3-41A8-A0B4-1FE716ABEFE3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93C7558B-A91F-4A35-B94E-E9BF71A53151}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -24217,4 +24261,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73E1A9BE-BAF3-41A8-A0B4-1FE716ABEFE3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>